<commit_message>
docs(sync): multi-source reconciliation model + L-037 root-cause correction + rc_out source-consistency guard
Introduce SYNC_RECONCILIATION_MODEL.md as the governing design for
multi-source sync integrity: no source is authoritative, extraction is
exact, cross-source diffs are human-arbitrated, and a run ends CLEAN or
DIFFS-PENDING (phased build R1-R5). Add the canonical "Sync Integrity —
Multi-Source Reconciliation" section to CLAUDE.md.

Rewrite L-037 in the learning ledger + rules digest: corrected root
cause to gsheet-sync Sheet-wins overwriting a correct proposed value
(audit-verified), with a pointer to the reconciliation model and a
Sheet-wins-retirement warning.

Keep the rc_out source-consistency guard as defense-in-depth across the
TS classifier, Python oracle, fixtures, specs, and tests. Vitest 304/304
pass, parity 12/12 clean.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/workers/sync/fixtures/rc_out/workbooks/rc_out_edge.xlsx
+++ b/workers/sync/fixtures/rc_out/workbooks/rc_out_edge.xlsx
@@ -453,7 +453,7 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>9999</v>
+        <v>1414</v>
       </c>
     </row>
     <row r="5">
@@ -546,7 +546,7 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>9999</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="13">

</xml_diff>